<commit_message>
Update model outputs 2026-10-10 22:22:58
</commit_message>
<xml_diff>
--- a/files/Straight_Greyhound_upcoming_rated_prices.xlsx
+++ b/files/Straight_Greyhound_upcoming_rated_prices.xlsx
@@ -203,7 +203,7 @@
     <t xml:space="preserve">Corey Mutton</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-11T12:07:00</t>
+    <t xml:space="preserve">2026-10-11T12:08:00</t>
   </si>
   <si>
     <t xml:space="preserve">6</t>
@@ -320,7 +320,7 @@
     <t xml:space="preserve">Claude Dacey</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-11T13:10:00</t>
+    <t xml:space="preserve">2026-10-11T13:07:00</t>
   </si>
   <si>
     <t xml:space="preserve">4</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-18 10:16:44
</commit_message>
<xml_diff>
--- a/files/Straight_Greyhound_upcoming_rated_prices.xlsx
+++ b/files/Straight_Greyhound_upcoming_rated_prices.xlsx
@@ -155,9 +155,6 @@
     <t xml:space="preserve">PROVISIONAL_OR_FINAL</t>
   </si>
   <si>
-    <t xml:space="preserve">BORN CHEEKY</t>
-  </si>
-  <si>
     <t xml:space="preserve">LIL MISS RIPLEY</t>
   </si>
   <si>
@@ -189,6 +186,9 @@
   </si>
   <si>
     <t xml:space="preserve">MOOSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AKULI HONEY</t>
   </si>
   <si>
     <t xml:space="preserve">BYE BRUNETTE</t>
@@ -2001,22 +2001,22 @@
         <v>44</v>
       </c>
       <c r="M2" t="n">
-        <v>1.99</v>
+        <v>1.6</v>
       </c>
       <c r="N2" t="n">
-        <v>1.96</v>
+        <v>1.66</v>
       </c>
       <c r="O2" t="n">
-        <v>2.5</v>
+        <v>1.89</v>
       </c>
       <c r="P2" t="n">
-        <v>1.28</v>
+        <v>1.16</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="R2" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="S2" t="n">
         <v>101.2</v>
@@ -2101,29 +2101,29 @@
       </c>
       <c r="I3"/>
       <c r="J3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K3" t="s">
         <v>47</v>
       </c>
       <c r="L3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="M3" t="n">
-        <v>4.9</v>
+        <v>5.72</v>
       </c>
       <c r="N3"/>
       <c r="O3" t="n">
-        <v>3.86</v>
+        <v>4.48</v>
       </c>
       <c r="P3" t="n">
-        <v>2.08</v>
+        <v>1.9</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.39</v>
+        <v>1.32</v>
       </c>
       <c r="R3" t="n">
-        <v>-1.3</v>
+        <v>-1.9</v>
       </c>
       <c r="S3"/>
       <c r="T3"/>
@@ -2194,64 +2194,80 @@
       </c>
       <c r="I4"/>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M4" t="n">
-        <v>7.02</v>
-      </c>
-      <c r="N4"/>
+        <v>14.62</v>
+      </c>
+      <c r="N4" t="n">
+        <v>11.46</v>
+      </c>
       <c r="O4" t="n">
-        <v>5.94</v>
+        <v>9.84</v>
       </c>
       <c r="P4" t="n">
-        <v>2.92</v>
+        <v>4.59</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.65</v>
+        <v>2.15</v>
       </c>
       <c r="R4" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="S4"/>
-      <c r="T4"/>
-      <c r="U4"/>
+        <v>-3.6</v>
+      </c>
+      <c r="S4" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="T4" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="U4" t="n">
+        <v>97.5</v>
+      </c>
       <c r="V4" t="n">
-        <v>100</v>
+        <v>102.7</v>
       </c>
       <c r="W4"/>
-      <c r="X4"/>
-      <c r="Y4"/>
-      <c r="Z4"/>
-      <c r="AA4"/>
+      <c r="X4" t="n">
+        <v>97.4</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>97.4</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>100.2</v>
+      </c>
       <c r="AB4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF4" t="n">
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH4" t="n">
         <v>0</v>
       </c>
       <c r="AI4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="AJ4" t="s">
         <v>46</v>
@@ -2287,80 +2303,80 @@
       </c>
       <c r="I5"/>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="M5" t="n">
-        <v>18.3</v>
+        <v>17.06</v>
       </c>
       <c r="N5" t="n">
-        <v>14.49</v>
+        <v>14.05</v>
       </c>
       <c r="O5" t="n">
-        <v>13.01</v>
+        <v>15.35</v>
       </c>
       <c r="P5" t="n">
-        <v>6.84</v>
+        <v>5.41</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.48</v>
+        <v>2.52</v>
       </c>
       <c r="R5" t="n">
-        <v>-3.6</v>
+        <v>-3.9</v>
       </c>
       <c r="S5" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="T5" t="n">
         <v>94.7</v>
       </c>
-      <c r="T5" t="n">
-        <v>94.8</v>
-      </c>
       <c r="U5" t="n">
-        <v>97.5</v>
+        <v>94.7</v>
       </c>
       <c r="V5" t="n">
-        <v>102.7</v>
+        <v>100</v>
       </c>
       <c r="W5"/>
       <c r="X5" t="n">
-        <v>97.4</v>
+        <v>94.8</v>
       </c>
       <c r="Y5" t="n">
-        <v>97.4</v>
+        <v>94.8</v>
       </c>
       <c r="Z5" t="n">
-        <v>94.8</v>
+        <v>94.7</v>
       </c>
       <c r="AA5" t="n">
-        <v>100.2</v>
+        <v>94.7</v>
       </c>
       <c r="AB5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AC5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AD5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AE5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AF5" t="n">
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AH5" t="n">
         <v>0</v>
       </c>
       <c r="AI5" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="AJ5" t="s">
         <v>46</v>
@@ -2396,80 +2412,74 @@
       </c>
       <c r="I6"/>
       <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" t="n">
+        <v>31.48</v>
+      </c>
+      <c r="N6" t="n">
+        <v>30.19</v>
+      </c>
+      <c r="O6" t="n">
+        <v>32.36</v>
+      </c>
+      <c r="P6" t="n">
+        <v>11.46</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-5.1</v>
+      </c>
+      <c r="S6" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="T6" t="n">
+        <v>90.9</v>
+      </c>
+      <c r="U6" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="V6" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="W6" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="X6"/>
+      <c r="Y6"/>
+      <c r="Z6"/>
+      <c r="AA6"/>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF6" t="n">
         <v>3</v>
       </c>
-      <c r="K6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L6" t="s">
-        <v>54</v>
-      </c>
-      <c r="M6" t="n">
-        <v>21.33</v>
-      </c>
-      <c r="N6" t="n">
-        <v>17.84</v>
-      </c>
-      <c r="O6" t="n">
-        <v>20.22</v>
-      </c>
-      <c r="P6" t="n">
-        <v>7.93</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="R6" t="n">
-        <v>-3.9</v>
-      </c>
-      <c r="S6" t="n">
-        <v>95.7</v>
-      </c>
-      <c r="T6" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="U6" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="V6" t="n">
-        <v>100</v>
-      </c>
-      <c r="W6"/>
-      <c r="X6" t="n">
-        <v>94.8</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>94.8</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>0</v>
-      </c>
       <c r="AG6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AH6" t="n">
         <v>0</v>
       </c>
       <c r="AI6" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="AJ6" t="s">
         <v>46</v>
@@ -2505,46 +2515,46 @@
       </c>
       <c r="I7"/>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K7" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" t="s">
         <v>55</v>
       </c>
-      <c r="L7" t="s">
-        <v>56</v>
-      </c>
       <c r="M7" t="n">
-        <v>36.77</v>
+        <v>58.96</v>
       </c>
       <c r="N7" t="n">
-        <v>32.89</v>
+        <v>65.32</v>
       </c>
       <c r="O7" t="n">
-        <v>42.55</v>
+        <v>47.77</v>
       </c>
       <c r="P7" t="n">
-        <v>15.64</v>
+        <v>22.06</v>
       </c>
       <c r="Q7" t="n">
-        <v>8.4</v>
+        <v>10.44</v>
       </c>
       <c r="R7" t="n">
-        <v>-5.1</v>
+        <v>-6.2</v>
       </c>
       <c r="S7" t="n">
-        <v>90.3</v>
+        <v>89.6</v>
       </c>
       <c r="T7" t="n">
-        <v>90.9</v>
+        <v>88.6</v>
       </c>
       <c r="U7" t="n">
-        <v>90.3</v>
+        <v>88</v>
       </c>
       <c r="V7" t="n">
-        <v>100.6</v>
+        <v>101.4</v>
       </c>
       <c r="W7" t="n">
-        <v>98.2</v>
+        <v>93.3</v>
       </c>
       <c r="X7"/>
       <c r="Y7"/>
@@ -2563,16 +2573,16 @@
         <v>5</v>
       </c>
       <c r="AF7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AH7" t="n">
         <v>0</v>
       </c>
       <c r="AI7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ7" t="s">
         <v>46</v>
@@ -2608,46 +2618,46 @@
       </c>
       <c r="I8"/>
       <c r="J8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K8" t="s">
         <v>58</v>
       </c>
       <c r="L8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M8" t="n">
-        <v>73.58</v>
+        <v>71.35</v>
       </c>
       <c r="N8" t="n">
-        <v>79.06</v>
+        <v>83.55</v>
       </c>
       <c r="O8" t="n">
-        <v>63.25</v>
+        <v>52.91</v>
       </c>
       <c r="P8" t="n">
-        <v>30.05</v>
+        <v>25.43</v>
       </c>
       <c r="Q8" t="n">
-        <v>15.88</v>
+        <v>11.96</v>
       </c>
       <c r="R8" t="n">
-        <v>-6.2</v>
+        <v>-6.3</v>
       </c>
       <c r="S8" t="n">
-        <v>89.6</v>
+        <v>86.4</v>
       </c>
       <c r="T8" t="n">
-        <v>88.6</v>
+        <v>86.4</v>
       </c>
       <c r="U8" t="n">
-        <v>88</v>
+        <v>85.8</v>
       </c>
       <c r="V8" t="n">
-        <v>101.4</v>
+        <v>100.3</v>
       </c>
       <c r="W8" t="n">
-        <v>93.3</v>
+        <v>94.5</v>
       </c>
       <c r="X8"/>
       <c r="Y8"/>
@@ -2663,19 +2673,19 @@
         <v>0</v>
       </c>
       <c r="AE8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AG8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AH8" t="n">
         <v>0</v>
       </c>
       <c r="AI8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ8" t="s">
         <v>46</v>
@@ -2720,19 +2730,19 @@
         <v>60</v>
       </c>
       <c r="M9" t="n">
-        <v>114.64</v>
+        <v>91.39</v>
       </c>
       <c r="N9" t="n">
-        <v>95.52</v>
+        <v>75.59</v>
       </c>
       <c r="O9" t="n">
-        <v>147.05</v>
+        <v>111.06</v>
       </c>
       <c r="P9" t="n">
-        <v>42.08</v>
+        <v>29.72</v>
       </c>
       <c r="Q9" t="n">
-        <v>20.13</v>
+        <v>13.11</v>
       </c>
       <c r="R9" t="n">
         <v>-6.9</v>
@@ -2786,7 +2796,7 @@
         <v>0</v>
       </c>
       <c r="AI9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ9" t="s">
         <v>46</v>
@@ -2937,22 +2947,22 @@
         <v>65</v>
       </c>
       <c r="L11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M11" t="n">
-        <v>7.34</v>
+        <v>7.32</v>
       </c>
       <c r="N11" t="n">
-        <v>7.16</v>
+        <v>7.13</v>
       </c>
       <c r="O11" t="n">
-        <v>6.67</v>
+        <v>6.65</v>
       </c>
       <c r="P11" t="n">
         <v>2.62</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.61</v>
+        <v>1.6</v>
       </c>
       <c r="R11" t="n">
         <v>-2.2</v>
@@ -3004,7 +3014,7 @@
         <v>0</v>
       </c>
       <c r="AI11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ11" t="s">
         <v>46</v>
@@ -3049,10 +3059,10 @@
         <v>67</v>
       </c>
       <c r="M12" t="n">
-        <v>9.61</v>
+        <v>9.59</v>
       </c>
       <c r="N12" t="n">
-        <v>9.54</v>
+        <v>9.52</v>
       </c>
       <c r="O12" t="n">
         <v>5.33</v>
@@ -3115,7 +3125,7 @@
         <v>0</v>
       </c>
       <c r="AI12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ12" t="s">
         <v>46</v>
@@ -3160,17 +3170,17 @@
         <v>69</v>
       </c>
       <c r="M13" t="n">
-        <v>11.81</v>
+        <v>11.82</v>
       </c>
       <c r="N13"/>
       <c r="O13" t="n">
-        <v>8.55</v>
+        <v>8.57</v>
       </c>
       <c r="P13" t="n">
-        <v>4.4</v>
+        <v>4.41</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.45</v>
+        <v>2.46</v>
       </c>
       <c r="R13" t="n">
         <v>-2.9</v>
@@ -3253,16 +3263,16 @@
         <v>71</v>
       </c>
       <c r="M14" t="n">
-        <v>24.42</v>
+        <v>24.35</v>
       </c>
       <c r="N14" t="n">
-        <v>25.81</v>
+        <v>25.8</v>
       </c>
       <c r="O14" t="n">
-        <v>12.56</v>
+        <v>12.52</v>
       </c>
       <c r="P14" t="n">
-        <v>8.31</v>
+        <v>8.29</v>
       </c>
       <c r="Q14" t="n">
         <v>4.23</v>
@@ -3319,7 +3329,7 @@
         <v>0</v>
       </c>
       <c r="AI14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ14" t="s">
         <v>46</v>
@@ -3364,19 +3374,19 @@
         <v>73</v>
       </c>
       <c r="M15" t="n">
-        <v>26.8</v>
+        <v>26.68</v>
       </c>
       <c r="N15" t="n">
-        <v>31.05</v>
+        <v>30.88</v>
       </c>
       <c r="O15" t="n">
-        <v>21.57</v>
+        <v>21.46</v>
       </c>
       <c r="P15" t="n">
-        <v>9.03</v>
+        <v>9</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.53</v>
+        <v>4.52</v>
       </c>
       <c r="R15" t="n">
         <v>-4.1</v>
@@ -3430,7 +3440,7 @@
         <v>0</v>
       </c>
       <c r="AI15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ15" t="s">
         <v>46</v>
@@ -3475,19 +3485,19 @@
         <v>75</v>
       </c>
       <c r="M16" t="n">
-        <v>144.14</v>
+        <v>144.22</v>
       </c>
       <c r="N16" t="n">
         <v>142.26</v>
       </c>
       <c r="O16" t="n">
-        <v>214.06</v>
+        <v>214.64</v>
       </c>
       <c r="P16" t="n">
-        <v>55.97</v>
+        <v>56.37</v>
       </c>
       <c r="Q16" t="n">
-        <v>28.19</v>
+        <v>28.28</v>
       </c>
       <c r="R16" t="n">
         <v>-7.3</v>
@@ -3541,7 +3551,7 @@
         <v>0</v>
       </c>
       <c r="AI16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ16" t="s">
         <v>46</v>
@@ -3586,19 +3596,19 @@
         <v>60</v>
       </c>
       <c r="M17" t="n">
-        <v>197.83</v>
+        <v>197.11</v>
       </c>
       <c r="N17" t="n">
-        <v>257.09</v>
+        <v>255.77</v>
       </c>
       <c r="O17" t="n">
-        <v>208.86</v>
+        <v>207.99</v>
       </c>
       <c r="P17" t="n">
-        <v>70.52</v>
+        <v>70.34</v>
       </c>
       <c r="Q17" t="n">
-        <v>34.16</v>
+        <v>34.09</v>
       </c>
       <c r="R17" t="n">
         <v>-7.1</v>
@@ -3652,7 +3662,7 @@
         <v>0</v>
       </c>
       <c r="AI17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ17" t="s">
         <v>46</v>
@@ -3700,7 +3710,7 @@
         <v>1.38</v>
       </c>
       <c r="N18" t="n">
-        <v>1.51</v>
+        <v>1.52</v>
       </c>
       <c r="O18" t="n">
         <v>1.32</v>
@@ -3712,7 +3722,7 @@
         <v>1.01</v>
       </c>
       <c r="R18" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="S18" t="n">
         <v>99.2</v>
@@ -3761,7 +3771,7 @@
         <v>0</v>
       </c>
       <c r="AI18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ18" t="s">
         <v>46</v>
@@ -3806,13 +3816,13 @@
         <v>83</v>
       </c>
       <c r="M19" t="n">
-        <v>4.66</v>
+        <v>4.64</v>
       </c>
       <c r="N19" t="n">
-        <v>3.87</v>
+        <v>3.86</v>
       </c>
       <c r="O19" t="n">
-        <v>5.43</v>
+        <v>5.4</v>
       </c>
       <c r="P19" t="n">
         <v>1.24</v>
@@ -3821,7 +3831,7 @@
         <v>1.04</v>
       </c>
       <c r="R19" t="n">
-        <v>-1.9</v>
+        <v>-1.8</v>
       </c>
       <c r="S19" t="n">
         <v>104.9</v>
@@ -3872,7 +3882,7 @@
         <v>1</v>
       </c>
       <c r="AI19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ19" t="s">
         <v>46</v>
@@ -3917,19 +3927,19 @@
         <v>75</v>
       </c>
       <c r="M20" t="n">
-        <v>38.31</v>
+        <v>38.13</v>
       </c>
       <c r="N20" t="n">
-        <v>29.9</v>
+        <v>29.83</v>
       </c>
       <c r="O20" t="n">
-        <v>43.71</v>
+        <v>43.53</v>
       </c>
       <c r="P20" t="n">
-        <v>9.49</v>
+        <v>9.47</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
       <c r="R20" t="n">
         <v>-4.9</v>
@@ -3983,7 +3993,7 @@
         <v>1</v>
       </c>
       <c r="AI20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ20" t="s">
         <v>46</v>
@@ -4028,19 +4038,19 @@
         <v>73</v>
       </c>
       <c r="M21" t="n">
-        <v>114.3</v>
+        <v>114.46</v>
       </c>
       <c r="N21" t="n">
         <v>60.65</v>
       </c>
       <c r="O21" t="n">
-        <v>102.28</v>
+        <v>102.43</v>
       </c>
       <c r="P21" t="n">
-        <v>25.19</v>
+        <v>25.26</v>
       </c>
       <c r="Q21" t="n">
-        <v>5.7</v>
+        <v>5.72</v>
       </c>
       <c r="R21" t="n">
         <v>-6.8</v>
@@ -4092,7 +4102,7 @@
         <v>0</v>
       </c>
       <c r="AI21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ21" t="s">
         <v>46</v>
@@ -4137,19 +4147,19 @@
         <v>87</v>
       </c>
       <c r="M22" t="n">
-        <v>116.35</v>
+        <v>116</v>
       </c>
       <c r="N22" t="n">
-        <v>109.3</v>
+        <v>109.06</v>
       </c>
       <c r="O22" t="n">
-        <v>145.03</v>
+        <v>144.3</v>
       </c>
       <c r="P22" t="n">
-        <v>30.15</v>
+        <v>30.11</v>
       </c>
       <c r="Q22" t="n">
-        <v>6.83</v>
+        <v>6.81</v>
       </c>
       <c r="R22" t="n">
         <v>-6.3</v>
@@ -4203,7 +4213,7 @@
         <v>0</v>
       </c>
       <c r="AI22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ22" t="s">
         <v>46</v>
@@ -4248,19 +4258,19 @@
         <v>71</v>
       </c>
       <c r="M23" t="n">
-        <v>120.79</v>
+        <v>121.1</v>
       </c>
       <c r="N23" t="n">
-        <v>77.34</v>
+        <v>77.46</v>
       </c>
       <c r="O23" t="n">
-        <v>167.19</v>
+        <v>167.47</v>
       </c>
       <c r="P23" t="n">
-        <v>29.11</v>
+        <v>29.25</v>
       </c>
       <c r="Q23" t="n">
-        <v>6.46</v>
+        <v>6.49</v>
       </c>
       <c r="R23" t="n">
         <v>-6.5</v>
@@ -4314,7 +4324,7 @@
         <v>0</v>
       </c>
       <c r="AI23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ23" t="s">
         <v>46</v>
@@ -4359,16 +4369,16 @@
         <v>90</v>
       </c>
       <c r="M24" t="n">
-        <v>139.08</v>
+        <v>139</v>
       </c>
       <c r="N24" t="n">
-        <v>109.3</v>
+        <v>109.06</v>
       </c>
       <c r="O24" t="n">
-        <v>90.89</v>
+        <v>90.66</v>
       </c>
       <c r="P24" t="n">
-        <v>33.94</v>
+        <v>33.98</v>
       </c>
       <c r="Q24" t="n">
         <v>7.43</v>
@@ -4425,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="AI24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ24" t="s">
         <v>46</v>
@@ -4536,7 +4546,7 @@
         <v>1</v>
       </c>
       <c r="AI25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ25" t="s">
         <v>46</v>
@@ -4581,16 +4591,16 @@
         <v>96</v>
       </c>
       <c r="M26" t="n">
-        <v>17.24</v>
+        <v>17.19</v>
       </c>
       <c r="N26" t="n">
-        <v>9.92</v>
+        <v>9.89</v>
       </c>
       <c r="O26" t="n">
-        <v>44.6</v>
+        <v>44.44</v>
       </c>
       <c r="P26" t="n">
-        <v>2.46</v>
+        <v>2.45</v>
       </c>
       <c r="Q26" t="n">
         <v>1.46</v>
@@ -4690,19 +4700,19 @@
         <v>90</v>
       </c>
       <c r="M27" t="n">
-        <v>31.79</v>
+        <v>31.93</v>
       </c>
       <c r="N27" t="n">
-        <v>23.13</v>
+        <v>23.24</v>
       </c>
       <c r="O27" t="n">
-        <v>36.08</v>
+        <v>36.22</v>
       </c>
       <c r="P27" t="n">
-        <v>3.63</v>
+        <v>3.64</v>
       </c>
       <c r="Q27" t="n">
-        <v>1.84</v>
+        <v>1.85</v>
       </c>
       <c r="R27" t="n">
         <v>-5.1</v>
@@ -4756,7 +4766,7 @@
         <v>0</v>
       </c>
       <c r="AI27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ27" t="s">
         <v>46</v>
@@ -4801,16 +4811,16 @@
         <v>99</v>
       </c>
       <c r="M28" t="n">
-        <v>49.73</v>
+        <v>49.66</v>
       </c>
       <c r="N28" t="n">
-        <v>35.2</v>
+        <v>35.1</v>
       </c>
       <c r="O28" t="n">
-        <v>113.82</v>
+        <v>113.62</v>
       </c>
       <c r="P28" t="n">
-        <v>5.82</v>
+        <v>5.81</v>
       </c>
       <c r="Q28" t="n">
         <v>2.67</v>
@@ -4867,7 +4877,7 @@
         <v>1</v>
       </c>
       <c r="AI28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ28" t="s">
         <v>46</v>
@@ -4912,19 +4922,19 @@
         <v>73</v>
       </c>
       <c r="M29" t="n">
-        <v>73.08</v>
+        <v>73.36</v>
       </c>
       <c r="N29" t="n">
-        <v>43.05</v>
+        <v>43.16</v>
       </c>
       <c r="O29" t="n">
-        <v>265.19</v>
+        <v>266.32</v>
       </c>
       <c r="P29" t="n">
-        <v>9.66</v>
+        <v>9.7</v>
       </c>
       <c r="Q29" t="n">
-        <v>4.12</v>
+        <v>4.13</v>
       </c>
       <c r="R29" t="n">
         <v>-6.9</v>
@@ -4976,7 +4986,7 @@
         <v>0</v>
       </c>
       <c r="AI29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ29" t="s">
         <v>46</v>
@@ -5021,19 +5031,19 @@
         <v>75</v>
       </c>
       <c r="M30" t="n">
-        <v>117.14</v>
+        <v>117</v>
       </c>
       <c r="N30" t="n">
-        <v>87.65</v>
+        <v>87.49</v>
       </c>
       <c r="O30" t="n">
-        <v>200.21</v>
+        <v>199.68</v>
       </c>
       <c r="P30" t="n">
-        <v>14.12</v>
+        <v>14.08</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.04</v>
+        <v>6.02</v>
       </c>
       <c r="R30" t="n">
         <v>-6.9</v>
@@ -5087,7 +5097,7 @@
         <v>1</v>
       </c>
       <c r="AI30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ30" t="s">
         <v>46</v>
@@ -5132,10 +5142,10 @@
         <v>105</v>
       </c>
       <c r="M31" t="n">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="N31" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
       <c r="O31" t="n">
         <v>2.61</v>
@@ -5196,7 +5206,7 @@
         <v>0</v>
       </c>
       <c r="AI31" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ31" t="s">
         <v>46</v>
@@ -5241,13 +5251,13 @@
         <v>96</v>
       </c>
       <c r="M32" t="n">
-        <v>3.97</v>
+        <v>3.98</v>
       </c>
       <c r="N32" t="n">
         <v>4.8</v>
       </c>
       <c r="O32" t="n">
-        <v>2.67</v>
+        <v>2.68</v>
       </c>
       <c r="P32" t="n">
         <v>1.96</v>
@@ -5299,7 +5309,7 @@
         <v>0</v>
       </c>
       <c r="AI32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ32" t="s">
         <v>46</v>
@@ -5344,19 +5354,19 @@
         <v>108</v>
       </c>
       <c r="M33" t="n">
-        <v>6.21</v>
+        <v>6.23</v>
       </c>
       <c r="N33" t="n">
-        <v>5.73</v>
+        <v>5.74</v>
       </c>
       <c r="O33" t="n">
-        <v>8.23</v>
+        <v>8.25</v>
       </c>
       <c r="P33" t="n">
-        <v>2.64</v>
+        <v>2.65</v>
       </c>
       <c r="Q33" t="n">
-        <v>1.57</v>
+        <v>1.58</v>
       </c>
       <c r="R33" t="n">
         <v>-1.4</v>
@@ -5408,7 +5418,7 @@
         <v>0</v>
       </c>
       <c r="AI33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ33" t="s">
         <v>46</v>
@@ -5453,19 +5463,19 @@
         <v>60</v>
       </c>
       <c r="M34" t="n">
-        <v>16.66</v>
+        <v>16.73</v>
       </c>
       <c r="N34" t="n">
-        <v>15.13</v>
+        <v>15.22</v>
       </c>
       <c r="O34" t="n">
-        <v>21.13</v>
+        <v>21.19</v>
       </c>
       <c r="P34" t="n">
-        <v>6.69</v>
+        <v>6.71</v>
       </c>
       <c r="Q34" t="n">
-        <v>3.51</v>
+        <v>3.52</v>
       </c>
       <c r="R34" t="n">
         <v>-2.7</v>
@@ -5519,7 +5529,7 @@
         <v>0</v>
       </c>
       <c r="AI34" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ34" t="s">
         <v>46</v>
@@ -5564,19 +5574,19 @@
         <v>111</v>
       </c>
       <c r="M35" t="n">
-        <v>23.7</v>
+        <v>23.64</v>
       </c>
       <c r="N35" t="n">
-        <v>22.24</v>
+        <v>22.2</v>
       </c>
       <c r="O35" t="n">
-        <v>20.34</v>
+        <v>20.29</v>
       </c>
       <c r="P35" t="n">
-        <v>9.11</v>
+        <v>9.08</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.55</v>
+        <v>4.54</v>
       </c>
       <c r="R35" t="n">
         <v>-3.2</v>
@@ -5628,7 +5638,7 @@
         <v>0</v>
       </c>
       <c r="AI35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ35" t="s">
         <v>46</v>
@@ -5673,19 +5683,19 @@
         <v>83</v>
       </c>
       <c r="M36" t="n">
-        <v>38.76</v>
+        <v>38.66</v>
       </c>
       <c r="N36" t="n">
-        <v>29.3</v>
+        <v>29.28</v>
       </c>
       <c r="O36" t="n">
-        <v>78.24</v>
+        <v>78.03</v>
       </c>
       <c r="P36" t="n">
-        <v>14.65</v>
+        <v>14.61</v>
       </c>
       <c r="Q36" t="n">
-        <v>7.17</v>
+        <v>7.15</v>
       </c>
       <c r="R36" t="n">
         <v>-4</v>
@@ -5739,7 +5749,7 @@
         <v>0</v>
       </c>
       <c r="AI36" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ36" t="s">
         <v>46</v>
@@ -5784,19 +5794,19 @@
         <v>114</v>
       </c>
       <c r="M37" t="n">
-        <v>77.14</v>
+        <v>77.12</v>
       </c>
       <c r="N37" t="n">
         <v>49.68</v>
       </c>
       <c r="O37" t="n">
-        <v>118.11</v>
+        <v>118</v>
       </c>
       <c r="P37" t="n">
-        <v>31.27</v>
+        <v>31.22</v>
       </c>
       <c r="Q37" t="n">
-        <v>15.49</v>
+        <v>15.46</v>
       </c>
       <c r="R37" t="n">
         <v>-5.2</v>
@@ -5848,7 +5858,7 @@
         <v>0</v>
       </c>
       <c r="AI37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ37" t="s">
         <v>46</v>
@@ -5893,19 +5903,19 @@
         <v>108</v>
       </c>
       <c r="M38" t="n">
-        <v>146.61</v>
+        <v>146.07</v>
       </c>
       <c r="N38" t="n">
-        <v>122.41</v>
+        <v>122.11</v>
       </c>
       <c r="O38" t="n">
-        <v>266.6</v>
+        <v>265.42</v>
       </c>
       <c r="P38" t="n">
-        <v>56.93</v>
+        <v>56.54</v>
       </c>
       <c r="Q38" t="n">
-        <v>27.16</v>
+        <v>27</v>
       </c>
       <c r="R38" t="n">
         <v>-5.7</v>
@@ -5957,7 +5967,7 @@
         <v>0</v>
       </c>
       <c r="AI38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ38" t="s">
         <v>46</v>
@@ -6008,7 +6018,7 @@
         <v>1.53</v>
       </c>
       <c r="O39" t="n">
-        <v>1.45</v>
+        <v>1.44</v>
       </c>
       <c r="P39" t="n">
         <v>1.14</v>
@@ -6066,7 +6076,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ39" t="s">
         <v>46</v>
@@ -6111,16 +6121,16 @@
         <v>122</v>
       </c>
       <c r="M40" t="n">
-        <v>6.66</v>
+        <v>6.64</v>
       </c>
       <c r="N40" t="n">
-        <v>6.28</v>
+        <v>6.27</v>
       </c>
       <c r="O40" t="n">
-        <v>11.35</v>
+        <v>11.33</v>
       </c>
       <c r="P40" t="n">
-        <v>2.22</v>
+        <v>2.21</v>
       </c>
       <c r="Q40" t="n">
         <v>1.44</v>
@@ -6175,7 +6185,7 @@
         <v>1</v>
       </c>
       <c r="AI40" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ40" t="s">
         <v>46</v>
@@ -6220,19 +6230,19 @@
         <v>124</v>
       </c>
       <c r="M41" t="n">
-        <v>16.28</v>
+        <v>16.34</v>
       </c>
       <c r="N41" t="n">
-        <v>19.27</v>
+        <v>19.32</v>
       </c>
       <c r="O41" t="n">
-        <v>10.84</v>
+        <v>10.88</v>
       </c>
       <c r="P41" t="n">
-        <v>5.02</v>
+        <v>5.04</v>
       </c>
       <c r="Q41" t="n">
-        <v>2.53</v>
+        <v>2.54</v>
       </c>
       <c r="R41" t="n">
         <v>-3.1</v>
@@ -6286,7 +6296,7 @@
         <v>0</v>
       </c>
       <c r="AI41" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ41" t="s">
         <v>46</v>
@@ -6331,19 +6341,19 @@
         <v>90</v>
       </c>
       <c r="M42" t="n">
-        <v>20.07</v>
+        <v>20.03</v>
       </c>
       <c r="N42" t="n">
-        <v>21.05</v>
+        <v>21.01</v>
       </c>
       <c r="O42" t="n">
-        <v>24.55</v>
+        <v>24.5</v>
       </c>
       <c r="P42" t="n">
-        <v>6.34</v>
+        <v>6.32</v>
       </c>
       <c r="Q42" t="n">
-        <v>3.18</v>
+        <v>3.17</v>
       </c>
       <c r="R42" t="n">
         <v>-3.5</v>
@@ -6397,7 +6407,7 @@
         <v>1</v>
       </c>
       <c r="AI42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ42" t="s">
         <v>46</v>
@@ -6442,19 +6452,19 @@
         <v>75</v>
       </c>
       <c r="M43" t="n">
-        <v>20.3</v>
+        <v>20.39</v>
       </c>
       <c r="N43" t="n">
-        <v>20.46</v>
+        <v>20.6</v>
       </c>
       <c r="O43" t="n">
-        <v>23.28</v>
+        <v>23.37</v>
       </c>
       <c r="P43" t="n">
-        <v>6.47</v>
+        <v>6.49</v>
       </c>
       <c r="Q43" t="n">
-        <v>3.25</v>
+        <v>3.26</v>
       </c>
       <c r="R43" t="n">
         <v>-3.5</v>
@@ -6508,7 +6518,7 @@
         <v>0</v>
       </c>
       <c r="AI43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ43" t="s">
         <v>46</v>
@@ -6553,19 +6563,19 @@
         <v>44</v>
       </c>
       <c r="M44" t="n">
-        <v>25.85</v>
+        <v>25.79</v>
       </c>
       <c r="N44" t="n">
-        <v>36.59</v>
+        <v>36.54</v>
       </c>
       <c r="O44" t="n">
-        <v>42.44</v>
+        <v>42.32</v>
       </c>
       <c r="P44" t="n">
-        <v>8.09</v>
+        <v>8.07</v>
       </c>
       <c r="Q44" t="n">
-        <v>3.89</v>
+        <v>3.88</v>
       </c>
       <c r="R44" t="n">
         <v>-3.6</v>
@@ -6619,7 +6629,7 @@
         <v>0</v>
       </c>
       <c r="AI44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ44" t="s">
         <v>46</v>
@@ -6664,19 +6674,19 @@
         <v>83</v>
       </c>
       <c r="M45" t="n">
-        <v>85.65</v>
+        <v>85.83</v>
       </c>
       <c r="N45" t="n">
-        <v>86.14</v>
+        <v>86.29</v>
       </c>
       <c r="O45" t="n">
-        <v>49.06</v>
+        <v>49.22</v>
       </c>
       <c r="P45" t="n">
-        <v>29.29</v>
+        <v>29.4</v>
       </c>
       <c r="Q45" t="n">
-        <v>14.29</v>
+        <v>14.33</v>
       </c>
       <c r="R45" t="n">
         <v>-5.7</v>
@@ -6779,7 +6789,7 @@
         <v>2.52</v>
       </c>
       <c r="O46" t="n">
-        <v>2.55</v>
+        <v>2.54</v>
       </c>
       <c r="P46" t="n">
         <v>1.47</v>
@@ -6837,7 +6847,7 @@
         <v>0</v>
       </c>
       <c r="AI46" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ46" t="s">
         <v>46</v>
@@ -6948,7 +6958,7 @@
         <v>1</v>
       </c>
       <c r="AI47" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ47" t="s">
         <v>46</v>
@@ -6993,13 +7003,13 @@
         <v>124</v>
       </c>
       <c r="M48" t="n">
-        <v>8.19</v>
+        <v>8.18</v>
       </c>
       <c r="N48" t="n">
-        <v>8.24</v>
+        <v>8.22</v>
       </c>
       <c r="O48" t="n">
-        <v>6.53</v>
+        <v>6.52</v>
       </c>
       <c r="P48" t="n">
         <v>3.62</v>
@@ -7059,7 +7069,7 @@
         <v>1</v>
       </c>
       <c r="AI48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ48" t="s">
         <v>46</v>
@@ -7104,16 +7114,16 @@
         <v>136</v>
       </c>
       <c r="M49" t="n">
-        <v>8.99</v>
+        <v>9.03</v>
       </c>
       <c r="N49" t="n">
-        <v>8.33</v>
+        <v>8.36</v>
       </c>
       <c r="O49" t="n">
-        <v>11.64</v>
+        <v>11.69</v>
       </c>
       <c r="P49" t="n">
-        <v>3.94</v>
+        <v>3.96</v>
       </c>
       <c r="Q49" t="n">
         <v>2.35</v>
@@ -7168,7 +7178,7 @@
         <v>0</v>
       </c>
       <c r="AI49" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ49" t="s">
         <v>46</v>
@@ -7213,19 +7223,19 @@
         <v>138</v>
       </c>
       <c r="M50" t="n">
-        <v>12.45</v>
+        <v>12.52</v>
       </c>
       <c r="N50" t="n">
-        <v>10.8</v>
+        <v>10.86</v>
       </c>
       <c r="O50" t="n">
-        <v>9.52</v>
+        <v>9.56</v>
       </c>
       <c r="P50" t="n">
-        <v>5.36</v>
+        <v>5.38</v>
       </c>
       <c r="Q50" t="n">
-        <v>3.08</v>
+        <v>3.09</v>
       </c>
       <c r="R50" t="n">
         <v>-2.3</v>
@@ -7277,7 +7287,7 @@
         <v>0</v>
       </c>
       <c r="AI50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ50" t="s">
         <v>46</v>
@@ -7322,22 +7332,22 @@
         <v>73</v>
       </c>
       <c r="M51" t="n">
-        <v>21.97</v>
+        <v>22</v>
       </c>
       <c r="N51" t="n">
-        <v>23</v>
+        <v>23.03</v>
       </c>
       <c r="O51" t="n">
-        <v>33.44</v>
+        <v>33.47</v>
       </c>
       <c r="P51" t="n">
         <v>9.09</v>
       </c>
       <c r="Q51" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="R51" t="n">
-        <v>-2.9</v>
+        <v>-3</v>
       </c>
       <c r="S51" t="n">
         <v>106.1</v>
@@ -7388,7 +7398,7 @@
         <v>0</v>
       </c>
       <c r="AI51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ51" t="s">
         <v>46</v>
@@ -7433,19 +7443,19 @@
         <v>124</v>
       </c>
       <c r="M52" t="n">
-        <v>41.44</v>
+        <v>41.62</v>
       </c>
       <c r="N52" t="n">
-        <v>48.38</v>
+        <v>48.48</v>
       </c>
       <c r="O52" t="n">
-        <v>40.04</v>
+        <v>40.23</v>
       </c>
       <c r="P52" t="n">
-        <v>17.66</v>
+        <v>17.74</v>
       </c>
       <c r="Q52" t="n">
-        <v>9.79</v>
+        <v>9.82</v>
       </c>
       <c r="R52" t="n">
         <v>-3.7</v>
@@ -7499,7 +7509,7 @@
         <v>0</v>
       </c>
       <c r="AI52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ52" t="s">
         <v>46</v>
@@ -7547,7 +7557,7 @@
         <v>1.2</v>
       </c>
       <c r="N53" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="O53" t="n">
         <v>1.17</v>
@@ -7559,7 +7569,7 @@
         <v>1.02</v>
       </c>
       <c r="R53" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="S53" t="n">
         <v>107.8</v>
@@ -7608,7 +7618,7 @@
         <v>0</v>
       </c>
       <c r="AI53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ53" t="s">
         <v>46</v>
@@ -7653,13 +7663,13 @@
         <v>94</v>
       </c>
       <c r="M54" t="n">
-        <v>19</v>
+        <v>19.11</v>
       </c>
       <c r="N54" t="n">
-        <v>15.04</v>
+        <v>15.09</v>
       </c>
       <c r="O54" t="n">
-        <v>23.18</v>
+        <v>23.31</v>
       </c>
       <c r="P54" t="n">
         <v>3.04</v>
@@ -7668,7 +7678,7 @@
         <v>1.73</v>
       </c>
       <c r="R54" t="n">
-        <v>-4.1</v>
+        <v>-4.2</v>
       </c>
       <c r="S54" t="n">
         <v>99.8</v>
@@ -7717,7 +7727,7 @@
         <v>0</v>
       </c>
       <c r="AI54" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ54" t="s">
         <v>46</v>
@@ -7762,16 +7772,16 @@
         <v>146</v>
       </c>
       <c r="M55" t="n">
-        <v>26.1</v>
+        <v>26.25</v>
       </c>
       <c r="N55" t="n">
-        <v>24.65</v>
+        <v>24.76</v>
       </c>
       <c r="O55" t="n">
-        <v>35.46</v>
+        <v>35.67</v>
       </c>
       <c r="P55" t="n">
-        <v>4.08</v>
+        <v>4.09</v>
       </c>
       <c r="Q55" t="n">
         <v>2.13</v>
@@ -7871,19 +7881,19 @@
         <v>44</v>
       </c>
       <c r="M56" t="n">
-        <v>34.16</v>
+        <v>34.36</v>
       </c>
       <c r="N56" t="n">
-        <v>25.69</v>
+        <v>25.82</v>
       </c>
       <c r="O56" t="n">
-        <v>38.26</v>
+        <v>38.5</v>
       </c>
       <c r="P56" t="n">
-        <v>5.47</v>
+        <v>5.48</v>
       </c>
       <c r="Q56" t="n">
-        <v>2.71</v>
+        <v>2.72</v>
       </c>
       <c r="R56" t="n">
         <v>-5</v>
@@ -7935,7 +7945,7 @@
         <v>0</v>
       </c>
       <c r="AI56" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ56" t="s">
         <v>46</v>
@@ -7980,19 +7990,19 @@
         <v>149</v>
       </c>
       <c r="M57" t="n">
-        <v>47.01</v>
+        <v>46.91</v>
       </c>
       <c r="N57" t="n">
-        <v>44.63</v>
+        <v>44.55</v>
       </c>
       <c r="O57" t="n">
-        <v>33.69</v>
+        <v>33.64</v>
       </c>
       <c r="P57" t="n">
-        <v>6.95</v>
+        <v>6.92</v>
       </c>
       <c r="Q57" t="n">
-        <v>3.29</v>
+        <v>3.28</v>
       </c>
       <c r="R57" t="n">
         <v>-5.2</v>
@@ -8044,7 +8054,7 @@
         <v>1</v>
       </c>
       <c r="AI57" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ57" t="s">
         <v>46</v>
@@ -8089,19 +8099,19 @@
         <v>151</v>
       </c>
       <c r="M58" t="n">
-        <v>59.36</v>
+        <v>59.32</v>
       </c>
       <c r="N58" t="n">
-        <v>51.42</v>
+        <v>51.47</v>
       </c>
       <c r="O58" t="n">
-        <v>65.47</v>
+        <v>65.49</v>
       </c>
       <c r="P58" t="n">
-        <v>9.96</v>
+        <v>9.92</v>
       </c>
       <c r="Q58" t="n">
-        <v>4.71</v>
+        <v>4.7</v>
       </c>
       <c r="R58" t="n">
         <v>-5.8</v>
@@ -8198,19 +8208,19 @@
         <v>73</v>
       </c>
       <c r="M59" t="n">
-        <v>156.94</v>
+        <v>157.22</v>
       </c>
       <c r="N59" t="n">
-        <v>106.05</v>
+        <v>106.28</v>
       </c>
       <c r="O59" t="n">
-        <v>411.88</v>
+        <v>412.72</v>
       </c>
       <c r="P59" t="n">
-        <v>27.16</v>
+        <v>27.11</v>
       </c>
       <c r="Q59" t="n">
-        <v>12.14</v>
+        <v>12.13</v>
       </c>
       <c r="R59" t="n">
         <v>-7.6</v>
@@ -8262,7 +8272,7 @@
         <v>0</v>
       </c>
       <c r="AI59" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ59" t="s">
         <v>46</v>
@@ -8371,7 +8381,7 @@
         <v>0</v>
       </c>
       <c r="AI60" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ60" t="s">
         <v>46</v>
@@ -8416,16 +8426,16 @@
         <v>105</v>
       </c>
       <c r="M61" t="n">
-        <v>20.25</v>
+        <v>20.27</v>
       </c>
       <c r="N61" t="n">
-        <v>18.31</v>
+        <v>18.33</v>
       </c>
       <c r="O61" t="n">
-        <v>13.08</v>
+        <v>13.09</v>
       </c>
       <c r="P61" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="Q61" t="n">
         <v>1.04</v>
@@ -8525,16 +8535,16 @@
         <v>158</v>
       </c>
       <c r="M62" t="n">
-        <v>73.28</v>
+        <v>72.64</v>
       </c>
       <c r="N62" t="n">
-        <v>73.48</v>
+        <v>72.73</v>
       </c>
       <c r="O62" t="n">
-        <v>25.57</v>
+        <v>25.39</v>
       </c>
       <c r="P62" t="n">
-        <v>4.4</v>
+        <v>4.37</v>
       </c>
       <c r="Q62" t="n">
         <v>1.21</v>
@@ -8591,7 +8601,7 @@
         <v>1</v>
       </c>
       <c r="AI62" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ62" t="s">
         <v>46</v>
@@ -8636,19 +8646,19 @@
         <v>114</v>
       </c>
       <c r="M63" t="n">
-        <v>417.69</v>
+        <v>415.81</v>
       </c>
       <c r="N63" t="n">
-        <v>283.3</v>
+        <v>281.7</v>
       </c>
       <c r="O63" t="n">
-        <v>214.21</v>
+        <v>213.13</v>
       </c>
       <c r="P63" t="n">
-        <v>32.36</v>
+        <v>32.24</v>
       </c>
       <c r="Q63" t="n">
-        <v>7.68</v>
+        <v>7.69</v>
       </c>
       <c r="R63" t="n">
         <v>-9.2</v>
@@ -8700,7 +8710,7 @@
         <v>1</v>
       </c>
       <c r="AI63" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ63" t="s">
         <v>46</v>
@@ -8745,19 +8755,19 @@
         <v>90</v>
       </c>
       <c r="M64" t="n">
-        <v>666.24</v>
+        <v>664.21</v>
       </c>
       <c r="N64" t="n">
         <v>591.75</v>
       </c>
       <c r="O64" t="n">
-        <v>273.54</v>
+        <v>271.9</v>
       </c>
       <c r="P64" t="n">
-        <v>49.11</v>
+        <v>48.86</v>
       </c>
       <c r="Q64" t="n">
-        <v>11.89</v>
+        <v>11.88</v>
       </c>
       <c r="R64" t="n">
         <v>-9.2</v>
@@ -8811,7 +8821,7 @@
         <v>1</v>
       </c>
       <c r="AI64" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ64" t="s">
         <v>46</v>
@@ -8969,7 +8979,7 @@
       </c>
       <c r="N66"/>
       <c r="O66" t="n">
-        <v>3.32</v>
+        <v>3.31</v>
       </c>
       <c r="P66" t="n">
         <v>2.06</v>
@@ -9058,16 +9068,16 @@
         <v>75</v>
       </c>
       <c r="M67" t="n">
-        <v>9.75</v>
+        <v>9.73</v>
       </c>
       <c r="N67" t="n">
-        <v>12.45</v>
+        <v>12.44</v>
       </c>
       <c r="O67" t="n">
-        <v>10.35</v>
+        <v>10.32</v>
       </c>
       <c r="P67" t="n">
-        <v>3.7</v>
+        <v>3.69</v>
       </c>
       <c r="Q67" t="n">
         <v>1.95</v>
@@ -9124,7 +9134,7 @@
         <v>1</v>
       </c>
       <c r="AI67" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ67" t="s">
         <v>46</v>
@@ -9169,19 +9179,19 @@
         <v>83</v>
       </c>
       <c r="M68" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="N68" t="n">
+        <v>9.04</v>
+      </c>
+      <c r="O68" t="n">
         <v>10.43</v>
       </c>
-      <c r="N68" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="O68" t="n">
-        <v>10.37</v>
-      </c>
       <c r="P68" t="n">
-        <v>3.8</v>
+        <v>3.81</v>
       </c>
       <c r="Q68" t="n">
-        <v>2.01</v>
+        <v>2.02</v>
       </c>
       <c r="R68" t="n">
         <v>-2.7</v>
@@ -9233,7 +9243,7 @@
         <v>0</v>
       </c>
       <c r="AI68" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ68" t="s">
         <v>46</v>
@@ -9278,16 +9288,16 @@
         <v>158</v>
       </c>
       <c r="M69" t="n">
-        <v>26.21</v>
+        <v>26.24</v>
       </c>
       <c r="N69" t="n">
-        <v>29.46</v>
+        <v>29.49</v>
       </c>
       <c r="O69" t="n">
-        <v>11.95</v>
+        <v>11.97</v>
       </c>
       <c r="P69" t="n">
-        <v>9.63</v>
+        <v>9.64</v>
       </c>
       <c r="Q69" t="n">
         <v>4.66</v>
@@ -9384,22 +9394,22 @@
         <v>167</v>
       </c>
       <c r="L70" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M70" t="n">
-        <v>45.54</v>
+        <v>45.71</v>
       </c>
       <c r="N70" t="n">
-        <v>57.51</v>
+        <v>57.77</v>
       </c>
       <c r="O70" t="n">
-        <v>35.24</v>
+        <v>35.41</v>
       </c>
       <c r="P70" t="n">
-        <v>18.19</v>
+        <v>18.26</v>
       </c>
       <c r="Q70" t="n">
-        <v>9.03</v>
+        <v>9.06</v>
       </c>
       <c r="R70" t="n">
         <v>-5.1</v>
@@ -9445,7 +9455,7 @@
         <v>0</v>
       </c>
       <c r="AI70" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ70" t="s">
         <v>46</v>
@@ -9556,7 +9566,7 @@
         <v>0</v>
       </c>
       <c r="AI71" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ71" t="s">
         <v>46</v>
@@ -10463,7 +10473,7 @@
         <v>1</v>
       </c>
       <c r="AI80" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ80" t="s">
         <v>46</v>
@@ -10574,7 +10584,7 @@
         <v>0</v>
       </c>
       <c r="AI81" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ81" t="s">
         <v>46</v>
@@ -10685,7 +10695,7 @@
         <v>0</v>
       </c>
       <c r="AI82" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ82" t="s">
         <v>46</v>
@@ -10796,7 +10806,7 @@
         <v>0</v>
       </c>
       <c r="AI83" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ83" t="s">
         <v>46</v>
@@ -10907,7 +10917,7 @@
         <v>0</v>
       </c>
       <c r="AI84" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ84" t="s">
         <v>46</v>
@@ -11129,7 +11139,7 @@
         <v>0</v>
       </c>
       <c r="AI86" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ86" t="s">
         <v>46</v>
@@ -11240,7 +11250,7 @@
         <v>0</v>
       </c>
       <c r="AI87" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ87" t="s">
         <v>46</v>
@@ -11351,7 +11361,7 @@
         <v>0</v>
       </c>
       <c r="AI88" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ88" t="s">
         <v>46</v>
@@ -11462,7 +11472,7 @@
         <v>0</v>
       </c>
       <c r="AI89" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ89" t="s">
         <v>46</v>
@@ -11573,7 +11583,7 @@
         <v>0</v>
       </c>
       <c r="AI90" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ90" t="s">
         <v>46</v>
@@ -11963,7 +11973,7 @@
         <v>0</v>
       </c>
       <c r="AI94" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ94" t="s">
         <v>46</v>
@@ -12171,7 +12181,7 @@
         <v>0</v>
       </c>
       <c r="AI96" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ96" t="s">
         <v>46</v>
@@ -12276,7 +12286,7 @@
         <v>0</v>
       </c>
       <c r="AI97" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ97" t="s">
         <v>46</v>
@@ -12387,7 +12397,7 @@
         <v>0</v>
       </c>
       <c r="AI98" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ98" t="s">
         <v>46</v>
@@ -12684,7 +12694,7 @@
         <v>0</v>
       </c>
       <c r="AI101" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ101" t="s">
         <v>46</v>
@@ -12795,7 +12805,7 @@
         <v>0</v>
       </c>
       <c r="AI102" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ102" t="s">
         <v>46</v>
@@ -12906,7 +12916,7 @@
         <v>0</v>
       </c>
       <c r="AI103" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ103" t="s">
         <v>46</v>
@@ -13017,7 +13027,7 @@
         <v>0</v>
       </c>
       <c r="AI104" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ104" t="s">
         <v>46</v>
@@ -13128,7 +13138,7 @@
         <v>0</v>
       </c>
       <c r="AI105" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ105" t="s">
         <v>46</v>
@@ -13344,7 +13354,7 @@
         <v>0</v>
       </c>
       <c r="AI107" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ107" t="s">
         <v>46</v>
@@ -13566,7 +13576,7 @@
         <v>0</v>
       </c>
       <c r="AI109" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ109" t="s">
         <v>46</v>
@@ -13788,7 +13798,7 @@
         <v>0</v>
       </c>
       <c r="AI111" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ111" t="s">
         <v>46</v>
@@ -13899,7 +13909,7 @@
         <v>0</v>
       </c>
       <c r="AI112" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ112" t="s">
         <v>46</v>
@@ -14010,7 +14020,7 @@
         <v>0</v>
       </c>
       <c r="AI113" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ113" t="s">
         <v>46</v>
@@ -14412,7 +14422,7 @@
         <v>0</v>
       </c>
       <c r="AI117" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ117" t="s">
         <v>46</v>
@@ -14634,7 +14644,7 @@
         <v>0</v>
       </c>
       <c r="AI119" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ119" t="s">
         <v>46</v>
@@ -14745,7 +14755,7 @@
         <v>0</v>
       </c>
       <c r="AI120" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ120" t="s">
         <v>46</v>
@@ -14856,7 +14866,7 @@
         <v>0</v>
       </c>
       <c r="AI121" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ121" t="s">
         <v>46</v>
@@ -14967,7 +14977,7 @@
         <v>0</v>
       </c>
       <c r="AI122" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ122" t="s">
         <v>46</v>
@@ -15393,7 +15403,7 @@
         <v>1</v>
       </c>
       <c r="AI126" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ126" t="s">
         <v>46</v>
@@ -15504,7 +15514,7 @@
         <v>1</v>
       </c>
       <c r="AI127" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ127" t="s">
         <v>46</v>
@@ -15615,7 +15625,7 @@
         <v>0</v>
       </c>
       <c r="AI128" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ128" t="s">
         <v>46</v>
@@ -15726,7 +15736,7 @@
         <v>0</v>
       </c>
       <c r="AI129" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ129" t="s">
         <v>46</v>
@@ -15837,7 +15847,7 @@
         <v>0</v>
       </c>
       <c r="AI130" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ130" t="s">
         <v>46</v>
@@ -15948,7 +15958,7 @@
         <v>0</v>
       </c>
       <c r="AI131" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ131" t="s">
         <v>46</v>
@@ -16059,7 +16069,7 @@
         <v>0</v>
       </c>
       <c r="AI132" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ132" t="s">
         <v>46</v>
@@ -16170,7 +16180,7 @@
         <v>0</v>
       </c>
       <c r="AI133" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ133" t="s">
         <v>46</v>
@@ -16281,7 +16291,7 @@
         <v>0</v>
       </c>
       <c r="AI134" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ134" t="s">
         <v>46</v>
@@ -16503,7 +16513,7 @@
         <v>0</v>
       </c>
       <c r="AI136" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ136" t="s">
         <v>46</v>
@@ -16614,7 +16624,7 @@
         <v>0</v>
       </c>
       <c r="AI137" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ137" t="s">
         <v>46</v>
@@ -16812,7 +16822,7 @@
         <v>0</v>
       </c>
       <c r="AI139" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ139" t="s">
         <v>46</v>
@@ -16923,7 +16933,7 @@
         <v>0</v>
       </c>
       <c r="AI140" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ140" t="s">
         <v>46</v>
@@ -17034,7 +17044,7 @@
         <v>0</v>
       </c>
       <c r="AI141" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ141" t="s">
         <v>46</v>
@@ -17145,7 +17155,7 @@
         <v>0</v>
       </c>
       <c r="AI142" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ142" t="s">
         <v>46</v>
@@ -17256,7 +17266,7 @@
         <v>0</v>
       </c>
       <c r="AI143" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ143" t="s">
         <v>46</v>
@@ -17367,7 +17377,7 @@
         <v>0</v>
       </c>
       <c r="AI144" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ144" t="s">
         <v>46</v>
@@ -17478,7 +17488,7 @@
         <v>0</v>
       </c>
       <c r="AI145" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ145" t="s">
         <v>46</v>
@@ -17589,7 +17599,7 @@
         <v>0</v>
       </c>
       <c r="AI146" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ146" t="s">
         <v>46</v>
@@ -17700,7 +17710,7 @@
         <v>0</v>
       </c>
       <c r="AI147" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ147" t="s">
         <v>46</v>
@@ -17811,7 +17821,7 @@
         <v>0</v>
       </c>
       <c r="AI148" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ148" t="s">
         <v>46</v>
@@ -17922,7 +17932,7 @@
         <v>0</v>
       </c>
       <c r="AI149" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ149" t="s">
         <v>46</v>
@@ -18144,7 +18154,7 @@
         <v>0</v>
       </c>
       <c r="AI151" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ151" t="s">
         <v>46</v>
@@ -18477,7 +18487,7 @@
         <v>0</v>
       </c>
       <c r="AI154" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ154" t="s">
         <v>46</v>
@@ -18582,7 +18592,7 @@
         <v>0</v>
       </c>
       <c r="AI155" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ155" t="s">
         <v>46</v>
@@ -18786,7 +18796,7 @@
         <v>0</v>
       </c>
       <c r="AI157" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ157" t="s">
         <v>46</v>
@@ -18897,7 +18907,7 @@
         <v>0</v>
       </c>
       <c r="AI158" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ158" t="s">
         <v>46</v>
@@ -19008,7 +19018,7 @@
         <v>0</v>
       </c>
       <c r="AI159" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ159" t="s">
         <v>46</v>
@@ -19119,7 +19129,7 @@
         <v>0</v>
       </c>
       <c r="AI160" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ160" t="s">
         <v>46</v>
@@ -19230,7 +19240,7 @@
         <v>0</v>
       </c>
       <c r="AI161" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ161" t="s">
         <v>46</v>
@@ -19341,7 +19351,7 @@
         <v>0</v>
       </c>
       <c r="AI162" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ162" t="s">
         <v>46</v>
@@ -19545,7 +19555,7 @@
         <v>0</v>
       </c>
       <c r="AI164" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ164" t="s">
         <v>46</v>
@@ -19656,7 +19666,7 @@
         <v>0</v>
       </c>
       <c r="AI165" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ165" t="s">
         <v>46</v>
@@ -19767,7 +19777,7 @@
         <v>0</v>
       </c>
       <c r="AI166" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ166" t="s">
         <v>46</v>
@@ -20100,7 +20110,7 @@
         <v>0</v>
       </c>
       <c r="AI169" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ169" t="s">
         <v>46</v>
@@ -20211,7 +20221,7 @@
         <v>0</v>
       </c>
       <c r="AI170" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ170" t="s">
         <v>46</v>
@@ -20322,7 +20332,7 @@
         <v>0</v>
       </c>
       <c r="AI171" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ171" t="s">
         <v>46</v>
@@ -20823,7 +20833,7 @@
         <v>0</v>
       </c>
       <c r="AI176" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ176" t="s">
         <v>46</v>
@@ -21366,7 +21376,7 @@
         <v>0</v>
       </c>
       <c r="AI181" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ181" t="s">
         <v>46</v>
@@ -21849,7 +21859,7 @@
         <v>0</v>
       </c>
       <c r="AI186" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ186" t="s">
         <v>46</v>
@@ -22071,7 +22081,7 @@
         <v>0</v>
       </c>
       <c r="AI188" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ188" t="s">
         <v>46</v>
@@ -22275,7 +22285,7 @@
         <v>0</v>
       </c>
       <c r="AI190" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ190" t="s">
         <v>46</v>
@@ -22487,7 +22497,7 @@
         <v>0</v>
       </c>
       <c r="AI192" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ192" t="s">
         <v>46</v>
@@ -22598,7 +22608,7 @@
         <v>0</v>
       </c>
       <c r="AI193" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ193" t="s">
         <v>46</v>
@@ -22709,7 +22719,7 @@
         <v>0</v>
       </c>
       <c r="AI194" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ194" t="s">
         <v>46</v>
@@ -22820,7 +22830,7 @@
         <v>0</v>
       </c>
       <c r="AI195" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ195" t="s">
         <v>46</v>
@@ -23141,7 +23151,7 @@
         <v>0</v>
       </c>
       <c r="AI198" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ198" t="s">
         <v>46</v>
@@ -23246,7 +23256,7 @@
         <v>0</v>
       </c>
       <c r="AI199" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ199" t="s">
         <v>46</v>
@@ -23351,7 +23361,7 @@
         <v>0</v>
       </c>
       <c r="AI200" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ200" t="s">
         <v>46</v>
@@ -23676,7 +23686,7 @@
         <v>0</v>
       </c>
       <c r="AI203" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ203" t="s">
         <v>46</v>
@@ -23787,7 +23797,7 @@
         <v>0</v>
       </c>
       <c r="AI204" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ204" t="s">
         <v>46</v>
@@ -23898,7 +23908,7 @@
         <v>0</v>
       </c>
       <c r="AI205" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ205" t="s">
         <v>46</v>
@@ -24003,7 +24013,7 @@
         <v>0</v>
       </c>
       <c r="AI206" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ206" t="s">
         <v>46</v>
@@ -24114,7 +24124,7 @@
         <v>0</v>
       </c>
       <c r="AI207" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ207" t="s">
         <v>46</v>
@@ -24225,7 +24235,7 @@
         <v>0</v>
       </c>
       <c r="AI208" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ208" t="s">
         <v>46</v>
@@ -24336,7 +24346,7 @@
         <v>0</v>
       </c>
       <c r="AI209" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ209" t="s">
         <v>46</v>
@@ -24441,7 +24451,7 @@
         <v>0</v>
       </c>
       <c r="AI210" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ210" t="s">
         <v>46</v>
@@ -24552,7 +24562,7 @@
         <v>0</v>
       </c>
       <c r="AI211" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ211" t="s">
         <v>46</v>
@@ -24663,7 +24673,7 @@
         <v>0</v>
       </c>
       <c r="AI212" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ212" t="s">
         <v>46</v>
@@ -25065,7 +25075,7 @@
         <v>0</v>
       </c>
       <c r="AI216" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ216" t="s">
         <v>46</v>
@@ -25176,7 +25186,7 @@
         <v>0</v>
       </c>
       <c r="AI217" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ217" t="s">
         <v>46</v>
@@ -25287,7 +25297,7 @@
         <v>0</v>
       </c>
       <c r="AI218" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ218" t="s">
         <v>46</v>
@@ -25398,7 +25408,7 @@
         <v>0</v>
       </c>
       <c r="AI219" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ219" t="s">
         <v>46</v>
@@ -25509,7 +25519,7 @@
         <v>0</v>
       </c>
       <c r="AI220" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ220" t="s">
         <v>46</v>
@@ -25935,7 +25945,7 @@
         <v>0</v>
       </c>
       <c r="AI224" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ224" t="s">
         <v>46</v>
@@ -26046,7 +26056,7 @@
         <v>0</v>
       </c>
       <c r="AI225" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ225" t="s">
         <v>46</v>
@@ -26258,7 +26268,7 @@
         <v>0</v>
       </c>
       <c r="AI227" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ227" t="s">
         <v>46</v>
@@ -26369,7 +26379,7 @@
         <v>0</v>
       </c>
       <c r="AI228" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ228" t="s">
         <v>46</v>
@@ -26573,7 +26583,7 @@
         <v>0</v>
       </c>
       <c r="AI230" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ230" t="s">
         <v>46</v>
@@ -26795,7 +26805,7 @@
         <v>0</v>
       </c>
       <c r="AI232" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ232" t="s">
         <v>46</v>
@@ -26906,7 +26916,7 @@
         <v>0</v>
       </c>
       <c r="AI233" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ233" t="s">
         <v>46</v>
@@ -27011,7 +27021,7 @@
         <v>0</v>
       </c>
       <c r="AI234" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ234" t="s">
         <v>46</v>
@@ -27122,7 +27132,7 @@
         <v>0</v>
       </c>
       <c r="AI235" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ235" t="s">
         <v>46</v>
@@ -27233,7 +27243,7 @@
         <v>0</v>
       </c>
       <c r="AI236" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ236" t="s">
         <v>46</v>
@@ -27455,7 +27465,7 @@
         <v>0</v>
       </c>
       <c r="AI238" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ238" t="s">
         <v>46</v>
@@ -27566,7 +27576,7 @@
         <v>0</v>
       </c>
       <c r="AI239" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ239" t="s">
         <v>46</v>
@@ -27677,7 +27687,7 @@
         <v>0</v>
       </c>
       <c r="AI240" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ240" t="s">
         <v>46</v>
@@ -27899,7 +27909,7 @@
         <v>0</v>
       </c>
       <c r="AI242" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ242" t="s">
         <v>46</v>
@@ -28010,7 +28020,7 @@
         <v>0</v>
       </c>
       <c r="AI243" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ243" t="s">
         <v>46</v>
@@ -28232,7 +28242,7 @@
         <v>0</v>
       </c>
       <c r="AI245" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ245" t="s">
         <v>46</v>
@@ -28634,7 +28644,7 @@
         <v>0</v>
       </c>
       <c r="AI249" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ249" t="s">
         <v>46</v>
@@ -28856,7 +28866,7 @@
         <v>0</v>
       </c>
       <c r="AI251" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ251" t="s">
         <v>46</v>
@@ -28967,7 +28977,7 @@
         <v>0</v>
       </c>
       <c r="AI252" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ252" t="s">
         <v>46</v>
@@ -29078,7 +29088,7 @@
         <v>0</v>
       </c>
       <c r="AI253" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ253" t="s">
         <v>46</v>
@@ -29300,7 +29310,7 @@
         <v>0</v>
       </c>
       <c r="AI255" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ255" t="s">
         <v>46</v>
@@ -29405,7 +29415,7 @@
         <v>0</v>
       </c>
       <c r="AI256" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ256" t="s">
         <v>46</v>
@@ -29516,7 +29526,7 @@
         <v>0</v>
       </c>
       <c r="AI257" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ257" t="s">
         <v>46</v>
@@ -29627,7 +29637,7 @@
         <v>0</v>
       </c>
       <c r="AI258" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ258" t="s">
         <v>46</v>
@@ -29738,7 +29748,7 @@
         <v>0</v>
       </c>
       <c r="AI259" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ259" t="s">
         <v>46</v>
@@ -29849,7 +29859,7 @@
         <v>0</v>
       </c>
       <c r="AI260" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AJ260" t="s">
         <v>46</v>

</xml_diff>